<commit_message>
agregando unidades de set blanco
</commit_message>
<xml_diff>
--- a/Inventario_CJ.xlsx
+++ b/Inventario_CJ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/463e7e6710c11b9a/Algoritmos/negocio de CJ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C328D3DC-9808-4210-AC1F-B1D3E5EE4C41}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45E0BC35-9221-4FEE-845C-F0EC1FDD3C3F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="464" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="464" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="46">
   <si>
     <t>Producto</t>
   </si>
@@ -124,9 +124,6 @@
   </si>
   <si>
     <t>Set corto Blanco + Beige</t>
-  </si>
-  <si>
-    <t>INAXISTENCIA</t>
   </si>
   <si>
     <t>XXL</t>
@@ -466,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -595,7 +592,6 @@
     <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1442,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E13" s="5">
         <v>47900</v>
@@ -1598,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E17" s="5">
         <v>25000</v>
@@ -2129,11 +2125,9 @@
         <v>12</v>
       </c>
       <c r="C31" s="32">
-        <v>0</v>
-      </c>
-      <c r="D31" s="31" t="s">
-        <v>15</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D31" s="31"/>
       <c r="E31" s="5">
         <v>25000</v>
       </c>
@@ -2150,15 +2144,15 @@
       </c>
       <c r="I31" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="J31" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="K31" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2169,11 +2163,9 @@
         <v>18</v>
       </c>
       <c r="C32" s="32">
-        <v>0</v>
-      </c>
-      <c r="D32" s="31" t="s">
-        <v>15</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D32" s="31"/>
       <c r="E32" s="5">
         <v>25000</v>
       </c>
@@ -2190,15 +2182,15 @@
       </c>
       <c r="I32" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>75000</v>
       </c>
       <c r="J32" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="K32" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2209,11 +2201,9 @@
         <v>16</v>
       </c>
       <c r="C33" s="32">
-        <v>0</v>
-      </c>
-      <c r="D33" s="31" t="s">
-        <v>15</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D33" s="31"/>
       <c r="E33" s="5">
         <v>25000</v>
       </c>
@@ -2230,15 +2220,15 @@
       </c>
       <c r="I33" s="6">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="J33" s="6">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>200000</v>
       </c>
       <c r="K33" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2327,9 +2317,7 @@
       <c r="C36" s="37">
         <v>0</v>
       </c>
-      <c r="D36" s="38" t="s">
-        <v>28</v>
-      </c>
+      <c r="D36" s="38"/>
       <c r="E36" s="5">
         <v>28373</v>
       </c>
@@ -2438,10 +2426,10 @@
         <v>27</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C39" s="37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" s="35"/>
       <c r="E39" s="5">
@@ -2460,15 +2448,15 @@
       </c>
       <c r="I39" s="6">
         <f t="shared" si="7"/>
-        <v>56746</v>
+        <v>85119</v>
       </c>
       <c r="J39" s="6">
         <f t="shared" si="8"/>
-        <v>170000</v>
+        <v>255000</v>
       </c>
       <c r="K39" s="6">
         <f t="shared" si="9"/>
-        <v>113254</v>
+        <v>169881</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2511,7 +2499,7 @@
     </row>
     <row r="41" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="39" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B41" s="40" t="s">
         <v>16</v>
@@ -2549,7 +2537,7 @@
     </row>
     <row r="42" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B42" s="42">
         <v>28</v>
@@ -2558,7 +2546,7 @@
         <v>0</v>
       </c>
       <c r="D42" s="43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E42" s="5">
         <v>31000</v>
@@ -2589,16 +2577,16 @@
     </row>
     <row r="43" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="B43" s="42" t="s">
-        <v>32</v>
-      </c>
       <c r="C43" s="42">
         <v>0</v>
       </c>
       <c r="D43" s="43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E43" s="5">
         <v>31000</v>
@@ -2629,16 +2617,16 @@
     </row>
     <row r="44" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B44" s="42" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C44" s="42">
         <v>0</v>
       </c>
       <c r="D44" s="43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E44" s="5">
         <v>31000</v>
@@ -2669,15 +2657,17 @@
     </row>
     <row r="45" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="42" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C45" s="42">
         <v>0</v>
       </c>
-      <c r="D45" s="43"/>
+      <c r="D45" s="43" t="s">
+        <v>45</v>
+      </c>
       <c r="E45" s="5">
         <v>31000</v>
       </c>
@@ -2706,16 +2696,18 @@
       </c>
     </row>
     <row r="46" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="71" t="s">
-        <v>31</v>
+      <c r="A46" s="70" t="s">
+        <v>30</v>
       </c>
       <c r="B46" s="42">
         <v>34</v>
       </c>
-      <c r="C46" s="79">
-        <v>0</v>
-      </c>
-      <c r="D46" s="44"/>
+      <c r="C46" s="78">
+        <v>0</v>
+      </c>
+      <c r="D46" s="43" t="s">
+        <v>45</v>
+      </c>
       <c r="E46" s="5">
         <v>31000</v>
       </c>
@@ -2744,17 +2736,17 @@
       </c>
     </row>
     <row r="47" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="74" t="s">
-        <v>35</v>
-      </c>
-      <c r="B47" s="45" t="s">
+      <c r="A47" s="73" t="s">
+        <v>34</v>
+      </c>
+      <c r="B47" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="45">
+      <c r="C47" s="44">
         <v>2</v>
       </c>
-      <c r="D47" s="75"/>
-      <c r="E47" s="70">
+      <c r="D47" s="74"/>
+      <c r="E47" s="69">
         <v>25000</v>
       </c>
       <c r="F47" s="5">
@@ -2782,17 +2774,17 @@
       </c>
     </row>
     <row r="48" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="74" t="s">
-        <v>35</v>
-      </c>
-      <c r="B48" s="45" t="s">
+      <c r="A48" s="73" t="s">
+        <v>34</v>
+      </c>
+      <c r="B48" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C48" s="45">
+      <c r="C48" s="44">
         <v>2</v>
       </c>
-      <c r="D48" s="46"/>
-      <c r="E48" s="70">
+      <c r="D48" s="45"/>
+      <c r="E48" s="69">
         <v>25000</v>
       </c>
       <c r="F48" s="5">
@@ -2820,19 +2812,19 @@
       </c>
     </row>
     <row r="49" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="74" t="s">
+      <c r="A49" s="73" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="44" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="77">
+        <v>3</v>
+      </c>
+      <c r="D49" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="B49" s="45" t="s">
-        <v>16</v>
-      </c>
-      <c r="C49" s="78">
-        <v>3</v>
-      </c>
-      <c r="D49" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="E49" s="70">
+      <c r="E49" s="69">
         <v>25000</v>
       </c>
       <c r="F49" s="5">
@@ -2860,17 +2852,17 @@
       </c>
     </row>
     <row r="50" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="74" t="s">
-        <v>35</v>
-      </c>
-      <c r="B50" s="76" t="s">
+      <c r="A50" s="73" t="s">
+        <v>34</v>
+      </c>
+      <c r="B50" s="75" t="s">
         <v>18</v>
       </c>
-      <c r="C50" s="76">
+      <c r="C50" s="75">
         <v>2</v>
       </c>
-      <c r="D50" s="77"/>
-      <c r="E50" s="70">
+      <c r="D50" s="76"/>
+      <c r="E50" s="69">
         <v>25000</v>
       </c>
       <c r="F50" s="5">
@@ -2898,17 +2890,17 @@
       </c>
     </row>
     <row r="51" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="80" t="s">
-        <v>45</v>
-      </c>
-      <c r="B51" s="81" t="s">
+      <c r="A51" s="79" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="C51" s="83">
+      <c r="C51" s="82">
         <v>2</v>
       </c>
-      <c r="D51" s="82"/>
-      <c r="E51" s="70">
+      <c r="D51" s="81"/>
+      <c r="E51" s="69">
         <v>20000</v>
       </c>
       <c r="F51" s="5">
@@ -2936,17 +2928,17 @@
       </c>
     </row>
     <row r="52" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="72" t="s">
-        <v>37</v>
-      </c>
-      <c r="B52" s="73" t="s">
+      <c r="A52" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="C52" s="73">
+      <c r="C52" s="72">
         <v>2</v>
       </c>
-      <c r="D52" s="72"/>
-      <c r="E52" s="70">
+      <c r="D52" s="71"/>
+      <c r="E52" s="69">
         <v>25000</v>
       </c>
       <c r="F52" s="5">
@@ -2974,17 +2966,17 @@
       </c>
     </row>
     <row r="53" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="B53" s="49" t="s">
+      <c r="A53" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="B53" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="C53" s="48">
+      <c r="C53" s="47">
         <v>2</v>
       </c>
-      <c r="D53" s="50"/>
-      <c r="E53" s="70">
+      <c r="D53" s="49"/>
+      <c r="E53" s="69">
         <v>25000</v>
       </c>
       <c r="F53" s="5">
@@ -3012,19 +3004,19 @@
       </c>
     </row>
     <row r="54" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="B54" s="49" t="s">
+      <c r="A54" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="B54" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="C54" s="48">
+      <c r="C54" s="47">
         <v>1</v>
       </c>
-      <c r="D54" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="E54" s="70">
+      <c r="D54" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54" s="69">
         <v>25000</v>
       </c>
       <c r="F54" s="5">
@@ -3052,19 +3044,19 @@
       </c>
     </row>
     <row r="55" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="47" t="s">
-        <v>37</v>
-      </c>
-      <c r="B55" s="48" t="s">
+      <c r="A55" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="B55" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C55" s="48">
-        <v>0</v>
-      </c>
-      <c r="D55" s="50" t="s">
-        <v>36</v>
-      </c>
-      <c r="E55" s="70">
+      <c r="C55" s="47">
+        <v>0</v>
+      </c>
+      <c r="D55" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55" s="69">
         <v>25000</v>
       </c>
       <c r="G55" s="6">
@@ -3089,17 +3081,17 @@
       </c>
     </row>
     <row r="56" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="B56" s="52">
+      <c r="A56" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B56" s="51">
         <v>28</v>
       </c>
-      <c r="C56" s="52">
-        <v>0</v>
-      </c>
-      <c r="D56" s="53" t="s">
-        <v>36</v>
+      <c r="C56" s="51">
+        <v>0</v>
+      </c>
+      <c r="D56" s="52" t="s">
+        <v>35</v>
       </c>
       <c r="E56" s="5">
         <v>26000</v>
@@ -3129,16 +3121,16 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" s="52" t="s">
-        <v>32</v>
-      </c>
-      <c r="C57" s="52">
+      <c r="A57" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B57" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57" s="51">
         <v>1</v>
       </c>
-      <c r="D57" s="53"/>
+      <c r="D57" s="52"/>
       <c r="E57" s="5">
         <v>26000</v>
       </c>
@@ -3167,16 +3159,16 @@
       </c>
     </row>
     <row r="58" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="52" t="s">
-        <v>33</v>
-      </c>
-      <c r="C58" s="52">
+      <c r="A58" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B58" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="C58" s="51">
         <v>1</v>
       </c>
-      <c r="D58" s="53"/>
+      <c r="D58" s="52"/>
       <c r="E58" s="5">
         <v>26000</v>
       </c>
@@ -3205,17 +3197,17 @@
       </c>
     </row>
     <row r="59" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="B59" s="54">
+      <c r="A59" s="50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B59" s="53">
         <v>32</v>
       </c>
-      <c r="C59" s="54">
-        <v>0</v>
-      </c>
-      <c r="D59" s="53" t="s">
-        <v>36</v>
+      <c r="C59" s="53">
+        <v>0</v>
+      </c>
+      <c r="D59" s="52" t="s">
+        <v>35</v>
       </c>
       <c r="E59" s="5">
         <v>26000</v>
@@ -3245,17 +3237,17 @@
       </c>
     </row>
     <row r="60" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="55" t="s">
-        <v>38</v>
-      </c>
-      <c r="B60" s="54">
+      <c r="A60" s="54" t="s">
+        <v>37</v>
+      </c>
+      <c r="B60" s="53">
         <v>34</v>
       </c>
-      <c r="C60" s="54">
-        <v>0</v>
-      </c>
-      <c r="D60" s="56" t="s">
-        <v>36</v>
+      <c r="C60" s="53">
+        <v>0</v>
+      </c>
+      <c r="D60" s="55" t="s">
+        <v>35</v>
       </c>
       <c r="E60" s="5">
         <v>26000</v>
@@ -3285,17 +3277,17 @@
       </c>
     </row>
     <row r="61" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="B61" s="58" t="s">
+      <c r="A61" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="60">
-        <v>0</v>
-      </c>
-      <c r="D61" s="59" t="s">
-        <v>36</v>
+      <c r="C61" s="59">
+        <v>0</v>
+      </c>
+      <c r="D61" s="58" t="s">
+        <v>35</v>
       </c>
       <c r="E61" s="5">
         <v>25000</v>
@@ -3325,16 +3317,16 @@
       </c>
     </row>
     <row r="62" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="B62" s="58" t="s">
+      <c r="A62" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B62" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C62" s="60">
+      <c r="C62" s="59">
         <v>1</v>
       </c>
-      <c r="D62" s="59"/>
+      <c r="D62" s="58"/>
       <c r="E62" s="5">
         <v>25000</v>
       </c>
@@ -3363,16 +3355,16 @@
       </c>
     </row>
     <row r="63" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="B63" s="58" t="s">
+      <c r="A63" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B63" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="C63" s="60">
+      <c r="C63" s="59">
         <v>2</v>
       </c>
-      <c r="D63" s="59"/>
+      <c r="D63" s="58"/>
       <c r="E63" s="5">
         <v>25000</v>
       </c>
@@ -3401,16 +3393,16 @@
       </c>
     </row>
     <row r="64" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="57" t="s">
-        <v>39</v>
-      </c>
-      <c r="B64" s="58" t="s">
+      <c r="A64" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="B64" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C64" s="60">
+      <c r="C64" s="59">
         <v>1</v>
       </c>
-      <c r="D64" s="57"/>
+      <c r="D64" s="56"/>
       <c r="E64" s="5">
         <v>25000</v>
       </c>
@@ -3439,36 +3431,36 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="61" t="s">
+      <c r="A65" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="B65" s="61"/>
+      <c r="C65" s="62">
+        <f>SUM(C2:C64)</f>
+        <v>80</v>
+      </c>
+      <c r="D65" s="61"/>
+      <c r="K65" s="63">
+        <f>SUM(K2:K64)</f>
+        <v>3979097</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="B65" s="62"/>
-      <c r="C65" s="63">
-        <f>SUM(C2:C64)</f>
-        <v>72</v>
-      </c>
-      <c r="D65" s="62"/>
-      <c r="K65" s="64">
-        <f>SUM(K2:K64)</f>
-        <v>3397470</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="65" t="s">
+      <c r="I67" s="63">
+        <f>SUM(I2:I64)</f>
+        <v>2095903</v>
+      </c>
+      <c r="J67" s="63">
+        <f>SUM(J2:J64)</f>
+        <v>6075000</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="65" t="s">
         <v>41</v>
-      </c>
-      <c r="I67" s="64">
-        <f>SUM(I2:I64)</f>
-        <v>1892530</v>
-      </c>
-      <c r="J67" s="64">
-        <f>SUM(J2:J64)</f>
-        <v>5290000</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="66" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -3493,17 +3485,17 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="68">
+      <c r="B2" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A2)</f>
         <v>7</v>
       </c>
@@ -3513,10 +3505,10 @@
       </c>
     </row>
     <row r="3" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="67" t="s">
+      <c r="A3" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="68">
+      <c r="B3" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A3)</f>
         <v>12</v>
       </c>
@@ -3526,10 +3518,10 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="68">
+      <c r="B4" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A4)</f>
         <v>3</v>
       </c>
@@ -3539,10 +3531,10 @@
       </c>
     </row>
     <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="66" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="68">
+      <c r="B5" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A5)</f>
         <v>2</v>
       </c>
@@ -3552,10 +3544,10 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="67" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="68">
+      <c r="A6" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="67">
         <f>SUMIFS(Inventario!C3:C65,Inventario!A3:A65,A6)</f>
         <v>2</v>
       </c>
@@ -3565,10 +3557,10 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="68">
+      <c r="B7" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A7)</f>
         <v>4</v>
       </c>
@@ -3578,10 +3570,10 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="68">
+      <c r="B8" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A8)</f>
         <v>2</v>
       </c>
@@ -3591,10 +3583,10 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="67" t="s">
+      <c r="A9" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="68">
+      <c r="B9" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A9)</f>
         <v>3</v>
       </c>
@@ -3604,10 +3596,10 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="67" t="s">
+      <c r="A10" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="68">
+      <c r="B10" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A10)</f>
         <v>2</v>
       </c>
@@ -3617,23 +3609,23 @@
       </c>
     </row>
     <row r="11" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="67" t="s">
+      <c r="A11" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="68">
+      <c r="B11" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A11)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C11" s="6">
         <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A11)</f>
-        <v>225000</v>
+        <v>750000</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="67" t="s">
+      <c r="A12" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="68">
+      <c r="B12" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A12)</f>
         <v>1</v>
       </c>
@@ -3643,23 +3635,23 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="67" t="s">
+      <c r="A13" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="68">
+      <c r="B13" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A13)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="6">
         <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A13)</f>
-        <v>566270</v>
+        <v>622897</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="67" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="68">
+      <c r="A14" s="66" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A14)</f>
         <v>1</v>
       </c>
@@ -3669,10 +3661,10 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="67" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="68">
+      <c r="A15" s="66" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A15)</f>
         <v>0</v>
       </c>
@@ -3682,10 +3674,10 @@
       </c>
     </row>
     <row r="16" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="67" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="68">
+      <c r="A16" s="66" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A16)</f>
         <v>9</v>
       </c>
@@ -3695,10 +3687,10 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="67" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="68">
+      <c r="A17" s="66" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A17)</f>
         <v>5</v>
       </c>
@@ -3708,10 +3700,10 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="67" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="68">
+      <c r="A18" s="66" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A18)</f>
         <v>2</v>
       </c>
@@ -3721,10 +3713,10 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="67" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="68">
+      <c r="A19" s="66" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="67">
         <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A19)</f>
         <v>4</v>
       </c>
@@ -3734,16 +3726,16 @@
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="61" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="63">
+      <c r="A20" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="62">
         <f>SUM(B2:B19)</f>
-        <v>72</v>
-      </c>
-      <c r="C20" s="69">
+        <v>80</v>
+      </c>
+      <c r="C20" s="68">
         <f>SUM(C2:C19)</f>
-        <v>3397470</v>
+        <v>3979097</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agregando pantalones blancos al inventario
</commit_message>
<xml_diff>
--- a/Inventario_CJ.xlsx
+++ b/Inventario_CJ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/463e7e6710c11b9a/Algoritmos/negocio de CJ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45E0BC35-9221-4FEE-845C-F0EC1FDD3C3F}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7147CD00-2E01-4A9F-9135-DD6FF5C83A0E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="464" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="48">
   <si>
     <t>Producto</t>
   </si>
@@ -178,6 +178,12 @@
   </si>
   <si>
     <t>VENDIDO</t>
+  </si>
+  <si>
+    <t>Pantalones Blancos</t>
+  </si>
+  <si>
+    <t>Mercancia no ha llegado</t>
   </si>
 </sst>
 </file>
@@ -260,7 +266,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -381,6 +387,12 @@
         <bgColor rgb="FF808000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor rgb="FF808000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -463,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -681,17 +693,23 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -957,7 +975,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" style="1" customWidth="1"/>
@@ -2249,23 +2267,23 @@
         <v>100000</v>
       </c>
       <c r="G34" s="6">
-        <f t="shared" ref="G34:G54" si="5">IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),F34-E34,"")</f>
+        <f t="shared" ref="G34:G59" si="5">IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),F34-E34,"")</f>
         <v>75000</v>
       </c>
       <c r="H34" s="7">
-        <f t="shared" ref="H34:H54" si="6">IF(AND(G34&lt;&gt;"",F34&lt;&gt;"",F34&lt;&gt;0),G34/F34,"")</f>
+        <f t="shared" ref="H34:H59" si="6">IF(AND(G34&lt;&gt;"",F34&lt;&gt;"",F34&lt;&gt;0),G34/F34,"")</f>
         <v>0.75</v>
       </c>
       <c r="I34" s="6">
-        <f t="shared" ref="I34:I64" si="7">IF(AND(C34&lt;&gt;"",E34&lt;&gt;""),C34*E34,"")</f>
+        <f t="shared" ref="I34:I69" si="7">IF(AND(C34&lt;&gt;"",E34&lt;&gt;""),C34*E34,"")</f>
         <v>75000</v>
       </c>
       <c r="J34" s="6">
-        <f t="shared" ref="J34:J64" si="8">IF(AND(C34&lt;&gt;"",F34&lt;&gt;""),C34*F34,"")</f>
+        <f t="shared" ref="J34:J69" si="8">IF(AND(C34&lt;&gt;"",F34&lt;&gt;""),C34*F34,"")</f>
         <v>300000</v>
       </c>
       <c r="K34" s="6">
-        <f t="shared" ref="K34:K64" si="9">IF(AND(C34&lt;&gt;"",G34&lt;&gt;""),C34*G34,"")</f>
+        <f t="shared" ref="K34:K69" si="9">IF(AND(C34&lt;&gt;"",G34&lt;&gt;""),C34*G34,"")</f>
         <v>225000</v>
       </c>
     </row>
@@ -2890,16 +2908,16 @@
       </c>
     </row>
     <row r="51" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="79" t="s">
+      <c r="A51" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="B51" s="80" t="s">
+      <c r="B51" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="C51" s="82">
+      <c r="C51" s="79">
         <v>2</v>
       </c>
-      <c r="D51" s="81"/>
+      <c r="D51" s="84"/>
       <c r="E51" s="69">
         <v>20000</v>
       </c>
@@ -2928,538 +2946,738 @@
       </c>
     </row>
     <row r="52" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="71" t="s">
-        <v>36</v>
-      </c>
-      <c r="B52" s="72" t="s">
-        <v>18</v>
-      </c>
-      <c r="C52" s="72">
-        <v>2</v>
-      </c>
-      <c r="D52" s="71"/>
+      <c r="A52" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B52" s="82">
+        <v>30</v>
+      </c>
+      <c r="C52" s="82">
+        <v>1</v>
+      </c>
+      <c r="D52" s="83" t="s">
+        <v>47</v>
+      </c>
       <c r="E52" s="69">
-        <v>25000</v>
+        <v>27978</v>
       </c>
       <c r="F52" s="5">
         <v>60000</v>
       </c>
       <c r="G52" s="6">
         <f t="shared" si="5"/>
+        <v>32022</v>
+      </c>
+      <c r="H52" s="7">
+        <f t="shared" ref="H52:H56" si="10">IF(AND(G52&lt;&gt;"",F52&lt;&gt;"",F52&lt;&gt;0),G52/F52,"")</f>
+        <v>0.53369999999999995</v>
+      </c>
+      <c r="I52" s="6">
+        <f t="shared" ref="I52:I56" si="11">IF(AND(C52&lt;&gt;"",E52&lt;&gt;""),C52*E52,"")</f>
+        <v>27978</v>
+      </c>
+      <c r="J52" s="6">
+        <f t="shared" ref="J52:J56" si="12">IF(AND(C52&lt;&gt;"",F52&lt;&gt;""),C52*F52,"")</f>
+        <v>60000</v>
+      </c>
+      <c r="K52" s="6">
+        <f t="shared" ref="K52:K56" si="13">IF(AND(C52&lt;&gt;"",G52&lt;&gt;""),C52*G52,"")</f>
+        <v>32022</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B53" s="82">
+        <v>31</v>
+      </c>
+      <c r="C53" s="82">
+        <v>1</v>
+      </c>
+      <c r="D53" s="83" t="s">
+        <v>47</v>
+      </c>
+      <c r="E53" s="69">
+        <v>27978</v>
+      </c>
+      <c r="F53" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G53" s="6">
+        <f t="shared" si="5"/>
+        <v>32022</v>
+      </c>
+      <c r="H53" s="7">
+        <f t="shared" si="10"/>
+        <v>0.53369999999999995</v>
+      </c>
+      <c r="I53" s="6">
+        <f t="shared" si="11"/>
+        <v>27978</v>
+      </c>
+      <c r="J53" s="6">
+        <f t="shared" si="12"/>
+        <v>60000</v>
+      </c>
+      <c r="K53" s="6">
+        <f t="shared" si="13"/>
+        <v>32022</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B54" s="82">
+        <v>32</v>
+      </c>
+      <c r="C54" s="82">
+        <v>1</v>
+      </c>
+      <c r="D54" s="83" t="s">
+        <v>47</v>
+      </c>
+      <c r="E54" s="69">
+        <v>27978</v>
+      </c>
+      <c r="F54" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G54" s="6">
+        <f t="shared" si="5"/>
+        <v>32022</v>
+      </c>
+      <c r="H54" s="7">
+        <f t="shared" si="10"/>
+        <v>0.53369999999999995</v>
+      </c>
+      <c r="I54" s="6">
+        <f t="shared" si="11"/>
+        <v>27978</v>
+      </c>
+      <c r="J54" s="6">
+        <f t="shared" si="12"/>
+        <v>60000</v>
+      </c>
+      <c r="K54" s="6">
+        <f t="shared" si="13"/>
+        <v>32022</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B55" s="82">
+        <v>34</v>
+      </c>
+      <c r="C55" s="82">
+        <v>1</v>
+      </c>
+      <c r="D55" s="83" t="s">
+        <v>47</v>
+      </c>
+      <c r="E55" s="69">
+        <v>27978</v>
+      </c>
+      <c r="F55" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G55" s="6">
+        <f t="shared" si="5"/>
+        <v>32022</v>
+      </c>
+      <c r="H55" s="7">
+        <f t="shared" si="10"/>
+        <v>0.53369999999999995</v>
+      </c>
+      <c r="I55" s="6">
+        <f t="shared" si="11"/>
+        <v>27978</v>
+      </c>
+      <c r="J55" s="6">
+        <f t="shared" si="12"/>
+        <v>60000</v>
+      </c>
+      <c r="K55" s="6">
+        <f t="shared" si="13"/>
+        <v>32022</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="81" t="s">
+        <v>46</v>
+      </c>
+      <c r="B56" s="82">
+        <v>36</v>
+      </c>
+      <c r="C56" s="82">
+        <v>1</v>
+      </c>
+      <c r="D56" s="83" t="s">
+        <v>47</v>
+      </c>
+      <c r="E56" s="69">
+        <v>27978</v>
+      </c>
+      <c r="F56" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G56" s="6">
+        <f t="shared" si="5"/>
+        <v>32022</v>
+      </c>
+      <c r="H56" s="7">
+        <f t="shared" si="10"/>
+        <v>0.53369999999999995</v>
+      </c>
+      <c r="I56" s="6">
+        <f t="shared" si="11"/>
+        <v>27978</v>
+      </c>
+      <c r="J56" s="6">
+        <f t="shared" si="12"/>
+        <v>60000</v>
+      </c>
+      <c r="K56" s="6">
+        <f t="shared" si="13"/>
+        <v>32022</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="B57" s="72" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" s="72">
+        <v>2</v>
+      </c>
+      <c r="D57" s="71"/>
+      <c r="E57" s="69">
+        <v>25000</v>
+      </c>
+      <c r="F57" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G57" s="6">
+        <f t="shared" si="5"/>
         <v>35000</v>
       </c>
-      <c r="H52" s="7">
+      <c r="H57" s="7">
         <f t="shared" si="6"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I52" s="6">
+      <c r="I57" s="6">
         <f t="shared" si="7"/>
         <v>50000</v>
       </c>
-      <c r="J52" s="6">
+      <c r="J57" s="6">
         <f t="shared" si="8"/>
         <v>120000</v>
       </c>
-      <c r="K52" s="6">
+      <c r="K57" s="6">
         <f t="shared" si="9"/>
         <v>70000</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="46" t="s">
+    <row r="58" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B53" s="48" t="s">
+      <c r="B58" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="C53" s="47">
+      <c r="C58" s="47">
         <v>2</v>
       </c>
-      <c r="D53" s="49"/>
-      <c r="E53" s="69">
-        <v>25000</v>
-      </c>
-      <c r="F53" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G53" s="6">
+      <c r="D58" s="49"/>
+      <c r="E58" s="69">
+        <v>25000</v>
+      </c>
+      <c r="F58" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G58" s="6">
         <f t="shared" si="5"/>
         <v>35000</v>
       </c>
-      <c r="H53" s="7">
+      <c r="H58" s="7">
         <f t="shared" si="6"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I53" s="6">
+      <c r="I58" s="6">
         <f t="shared" si="7"/>
         <v>50000</v>
       </c>
-      <c r="J53" s="6">
+      <c r="J58" s="6">
         <f t="shared" si="8"/>
         <v>120000</v>
       </c>
-      <c r="K53" s="6">
+      <c r="K58" s="6">
         <f t="shared" si="9"/>
         <v>70000</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="46" t="s">
+    <row r="59" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B54" s="48" t="s">
+      <c r="B59" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="C54" s="47">
+      <c r="C59" s="47">
         <v>1</v>
       </c>
-      <c r="D54" s="49" t="s">
+      <c r="D59" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E54" s="69">
-        <v>25000</v>
-      </c>
-      <c r="F54" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G54" s="6">
+      <c r="E59" s="69">
+        <v>25000</v>
+      </c>
+      <c r="F59" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G59" s="6">
         <f t="shared" si="5"/>
         <v>35000</v>
       </c>
-      <c r="H54" s="7">
+      <c r="H59" s="7">
         <f t="shared" si="6"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I54" s="6">
+      <c r="I59" s="6">
         <f t="shared" si="7"/>
         <v>25000</v>
       </c>
-      <c r="J54" s="6">
+      <c r="J59" s="6">
         <f t="shared" si="8"/>
         <v>60000</v>
       </c>
-      <c r="K54" s="6">
+      <c r="K59" s="6">
         <f t="shared" si="9"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="46" t="s">
+    <row r="60" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="B55" s="47" t="s">
+      <c r="B60" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C55" s="47">
-        <v>0</v>
-      </c>
-      <c r="D55" s="49" t="s">
+      <c r="C60" s="47">
+        <v>0</v>
+      </c>
+      <c r="D60" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E55" s="69">
-        <v>25000</v>
-      </c>
-      <c r="G55" s="6">
-        <f t="shared" ref="G55:G61" si="10">IF(AND(E55&lt;&gt;"",F56&lt;&gt;""),F56-E55,"")</f>
+      <c r="E60" s="69">
+        <v>25000</v>
+      </c>
+      <c r="G60" s="6">
+        <f t="shared" ref="G60:G66" si="14">IF(AND(E60&lt;&gt;"",F61&lt;&gt;""),F61-E60,"")</f>
         <v>35000</v>
       </c>
-      <c r="H55" s="7">
-        <f t="shared" ref="H55:H61" si="11">IF(AND(G55&lt;&gt;"",F56&lt;&gt;"",F56&lt;&gt;0),G55/F56,"")</f>
+      <c r="H60" s="7">
+        <f t="shared" ref="H60:H66" si="15">IF(AND(G60&lt;&gt;"",F61&lt;&gt;"",F61&lt;&gt;0),G60/F61,"")</f>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I55" s="6">
+      <c r="I60" s="6">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J55" s="6">
-        <f t="shared" ref="J55:J61" si="12">IF(AND(C55&lt;&gt;"",F56&lt;&gt;""),C55*F56,"")</f>
-        <v>0</v>
-      </c>
-      <c r="K55" s="6">
+      <c r="J60" s="6">
+        <f t="shared" ref="J60:J66" si="16">IF(AND(C60&lt;&gt;"",F61&lt;&gt;""),C60*F61,"")</f>
+        <v>0</v>
+      </c>
+      <c r="K60" s="6">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="50" t="s">
+    <row r="61" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="B56" s="51">
+      <c r="B61" s="51">
         <v>28</v>
       </c>
-      <c r="C56" s="51">
-        <v>0</v>
-      </c>
-      <c r="D56" s="52" t="s">
+      <c r="C61" s="51">
+        <v>0</v>
+      </c>
+      <c r="D61" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="E56" s="5">
+      <c r="E61" s="5">
         <v>26000</v>
       </c>
-      <c r="F56" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G56" s="6">
-        <f t="shared" si="10"/>
+      <c r="F61" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G61" s="6">
+        <f t="shared" si="14"/>
         <v>34000</v>
       </c>
-      <c r="H56" s="7">
-        <f t="shared" si="11"/>
+      <c r="H61" s="7">
+        <f t="shared" si="15"/>
         <v>0.56666666666666665</v>
       </c>
-      <c r="I56" s="6">
+      <c r="I61" s="6">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J56" s="6">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K56" s="6">
+      <c r="J61" s="6">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="K61" s="6">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="50" t="s">
+    <row r="62" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="51" t="s">
+      <c r="B62" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C57" s="51">
+      <c r="C62" s="51">
         <v>1</v>
       </c>
-      <c r="D57" s="52"/>
-      <c r="E57" s="5">
+      <c r="D62" s="52"/>
+      <c r="E62" s="5">
         <v>26000</v>
       </c>
-      <c r="F57" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G57" s="6">
-        <f t="shared" si="10"/>
+      <c r="F62" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G62" s="6">
+        <f t="shared" si="14"/>
         <v>34000</v>
       </c>
-      <c r="H57" s="7">
-        <f t="shared" si="11"/>
+      <c r="H62" s="7">
+        <f t="shared" si="15"/>
         <v>0.56666666666666665</v>
       </c>
-      <c r="I57" s="6">
+      <c r="I62" s="6">
         <f t="shared" si="7"/>
         <v>26000</v>
       </c>
-      <c r="J57" s="6">
-        <f t="shared" si="12"/>
-        <v>60000</v>
-      </c>
-      <c r="K57" s="6">
+      <c r="J62" s="6">
+        <f t="shared" si="16"/>
+        <v>60000</v>
+      </c>
+      <c r="K62" s="6">
         <f t="shared" si="9"/>
         <v>34000</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="50" t="s">
+    <row r="63" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="51" t="s">
+      <c r="B63" s="51" t="s">
         <v>32</v>
       </c>
-      <c r="C58" s="51">
+      <c r="C63" s="51">
         <v>1</v>
       </c>
-      <c r="D58" s="52"/>
-      <c r="E58" s="5">
+      <c r="D63" s="52"/>
+      <c r="E63" s="5">
         <v>26000</v>
       </c>
-      <c r="F58" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G58" s="6">
-        <f t="shared" si="10"/>
+      <c r="F63" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G63" s="6">
+        <f t="shared" si="14"/>
         <v>34000</v>
       </c>
-      <c r="H58" s="7">
-        <f t="shared" si="11"/>
+      <c r="H63" s="7">
+        <f t="shared" si="15"/>
         <v>0.56666666666666665</v>
       </c>
-      <c r="I58" s="6">
+      <c r="I63" s="6">
         <f t="shared" si="7"/>
         <v>26000</v>
       </c>
-      <c r="J58" s="6">
-        <f t="shared" si="12"/>
-        <v>60000</v>
-      </c>
-      <c r="K58" s="6">
+      <c r="J63" s="6">
+        <f t="shared" si="16"/>
+        <v>60000</v>
+      </c>
+      <c r="K63" s="6">
         <f t="shared" si="9"/>
         <v>34000</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="50" t="s">
+    <row r="64" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="B59" s="53">
+      <c r="B64" s="53">
         <v>32</v>
       </c>
-      <c r="C59" s="53">
-        <v>0</v>
-      </c>
-      <c r="D59" s="52" t="s">
+      <c r="C64" s="53">
+        <v>0</v>
+      </c>
+      <c r="D64" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="E59" s="5">
+      <c r="E64" s="5">
         <v>26000</v>
       </c>
-      <c r="F59" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G59" s="6">
-        <f t="shared" si="10"/>
+      <c r="F64" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G64" s="6">
+        <f t="shared" si="14"/>
         <v>34000</v>
       </c>
-      <c r="H59" s="7">
-        <f t="shared" si="11"/>
+      <c r="H64" s="7">
+        <f t="shared" si="15"/>
         <v>0.56666666666666665</v>
       </c>
-      <c r="I59" s="6">
+      <c r="I64" s="6">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J59" s="6">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K59" s="6">
+      <c r="J64" s="6">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="K64" s="6">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="54" t="s">
+    <row r="65" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="B60" s="53">
+      <c r="B65" s="53">
         <v>34</v>
       </c>
-      <c r="C60" s="53">
-        <v>0</v>
-      </c>
-      <c r="D60" s="55" t="s">
+      <c r="C65" s="53">
+        <v>0</v>
+      </c>
+      <c r="D65" s="55" t="s">
         <v>35</v>
       </c>
-      <c r="E60" s="5">
+      <c r="E65" s="5">
         <v>26000</v>
       </c>
-      <c r="F60" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G60" s="6">
-        <f t="shared" si="10"/>
+      <c r="F65" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G65" s="6">
+        <f t="shared" si="14"/>
         <v>34000</v>
       </c>
-      <c r="H60" s="7">
-        <f t="shared" si="11"/>
+      <c r="H65" s="7">
+        <f t="shared" si="15"/>
         <v>0.56666666666666665</v>
       </c>
-      <c r="I60" s="6">
+      <c r="I65" s="6">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J60" s="6">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K60" s="6">
+      <c r="J65" s="6">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="K65" s="6">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="56" t="s">
+    <row r="66" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="57" t="s">
+      <c r="B66" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="59">
-        <v>0</v>
-      </c>
-      <c r="D61" s="58" t="s">
+      <c r="C66" s="59">
+        <v>0</v>
+      </c>
+      <c r="D66" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="E61" s="5">
-        <v>25000</v>
-      </c>
-      <c r="F61" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G61" s="6">
-        <f t="shared" si="10"/>
+      <c r="E66" s="5">
+        <v>25000</v>
+      </c>
+      <c r="F66" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G66" s="6">
+        <f t="shared" si="14"/>
         <v>35000</v>
       </c>
-      <c r="H61" s="7">
-        <f t="shared" si="11"/>
+      <c r="H66" s="7">
+        <f t="shared" si="15"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I61" s="6">
+      <c r="I66" s="6">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="J61" s="6">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="K61" s="6">
+      <c r="J66" s="6">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="K66" s="6">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="56" t="s">
+    <row r="67" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="57" t="s">
+      <c r="B67" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="C62" s="59">
+      <c r="C67" s="59">
         <v>1</v>
       </c>
-      <c r="D62" s="58"/>
-      <c r="E62" s="5">
-        <v>25000</v>
-      </c>
-      <c r="F62" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G62" s="6">
-        <f t="shared" ref="G62:G64" si="13">IF(AND(E62&lt;&gt;"",F62&lt;&gt;""),F62-E62,"")</f>
+      <c r="D67" s="58"/>
+      <c r="E67" s="5">
+        <v>25000</v>
+      </c>
+      <c r="F67" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G67" s="6">
+        <f t="shared" ref="G67:G69" si="17">IF(AND(E67&lt;&gt;"",F67&lt;&gt;""),F67-E67,"")</f>
         <v>35000</v>
       </c>
-      <c r="H62" s="7">
-        <f t="shared" ref="H62:H64" si="14">IF(AND(G62&lt;&gt;"",F62&lt;&gt;"",F62&lt;&gt;0),G62/F62,"")</f>
+      <c r="H67" s="7">
+        <f t="shared" ref="H67:H69" si="18">IF(AND(G67&lt;&gt;"",F67&lt;&gt;"",F67&lt;&gt;0),G67/F67,"")</f>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I62" s="6">
+      <c r="I67" s="6">
         <f t="shared" si="7"/>
         <v>25000</v>
       </c>
-      <c r="J62" s="6">
+      <c r="J67" s="6">
         <f t="shared" si="8"/>
         <v>60000</v>
       </c>
-      <c r="K62" s="6">
+      <c r="K67" s="6">
         <f t="shared" si="9"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="56" t="s">
+    <row r="68" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B63" s="57" t="s">
+      <c r="B68" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="C63" s="59">
+      <c r="C68" s="59">
         <v>2</v>
       </c>
-      <c r="D63" s="58"/>
-      <c r="E63" s="5">
-        <v>25000</v>
-      </c>
-      <c r="F63" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G63" s="6">
-        <f t="shared" si="13"/>
+      <c r="D68" s="58"/>
+      <c r="E68" s="5">
+        <v>25000</v>
+      </c>
+      <c r="F68" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G68" s="6">
+        <f t="shared" si="17"/>
         <v>35000</v>
       </c>
-      <c r="H63" s="7">
-        <f t="shared" si="14"/>
+      <c r="H68" s="7">
+        <f t="shared" si="18"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I63" s="6">
+      <c r="I68" s="6">
         <f t="shared" si="7"/>
         <v>50000</v>
       </c>
-      <c r="J63" s="6">
+      <c r="J68" s="6">
         <f t="shared" si="8"/>
         <v>120000</v>
       </c>
-      <c r="K63" s="6">
+      <c r="K68" s="6">
         <f t="shared" si="9"/>
         <v>70000</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="56" t="s">
+    <row r="69" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B64" s="57" t="s">
+      <c r="B69" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C64" s="59">
+      <c r="C69" s="59">
         <v>1</v>
       </c>
-      <c r="D64" s="56"/>
-      <c r="E64" s="5">
-        <v>25000</v>
-      </c>
-      <c r="F64" s="5">
-        <v>60000</v>
-      </c>
-      <c r="G64" s="6">
-        <f t="shared" si="13"/>
+      <c r="D69" s="56"/>
+      <c r="E69" s="5">
+        <v>25000</v>
+      </c>
+      <c r="F69" s="5">
+        <v>60000</v>
+      </c>
+      <c r="G69" s="6">
+        <f t="shared" si="17"/>
         <v>35000</v>
       </c>
-      <c r="H64" s="7">
-        <f t="shared" si="14"/>
+      <c r="H69" s="7">
+        <f t="shared" si="18"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="I64" s="6">
+      <c r="I69" s="6">
         <f t="shared" si="7"/>
         <v>25000</v>
       </c>
-      <c r="J64" s="6">
+      <c r="J69" s="6">
         <f t="shared" si="8"/>
         <v>60000</v>
       </c>
-      <c r="K64" s="6">
+      <c r="K69" s="6">
         <f t="shared" si="9"/>
         <v>35000</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="60" t="s">
+    <row r="70" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="B65" s="61"/>
-      <c r="C65" s="62">
-        <f>SUM(C2:C64)</f>
-        <v>80</v>
-      </c>
-      <c r="D65" s="61"/>
-      <c r="K65" s="63">
-        <f>SUM(K2:K64)</f>
-        <v>3979097</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="64" t="s">
+      <c r="B70" s="61"/>
+      <c r="C70" s="62">
+        <f>SUM(C2:C69)</f>
+        <v>85</v>
+      </c>
+      <c r="D70" s="61"/>
+      <c r="K70" s="63">
+        <f>SUM(K2:K69)</f>
+        <v>4139207</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="I67" s="63">
-        <f>SUM(I2:I64)</f>
-        <v>2095903</v>
-      </c>
-      <c r="J67" s="63">
-        <f>SUM(J2:J64)</f>
-        <v>6075000</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="65" t="s">
+      <c r="I72" s="63">
+        <f>SUM(I2:I69)</f>
+        <v>2235793</v>
+      </c>
+      <c r="J72" s="63">
+        <f>SUM(J2:J69)</f>
+        <v>6375000</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" s="65" t="s">
         <v>41</v>
       </c>
     </row>
@@ -3496,11 +3714,11 @@
         <v>11</v>
       </c>
       <c r="B2" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A2)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A2)</f>
         <v>7</v>
       </c>
       <c r="C2" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A2)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A2)</f>
         <v>245000</v>
       </c>
     </row>
@@ -3509,11 +3727,11 @@
         <v>17</v>
       </c>
       <c r="B3" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A3)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A3)</f>
         <v>12</v>
       </c>
       <c r="C3" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A3)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A3)</f>
         <v>420000</v>
       </c>
     </row>
@@ -3522,11 +3740,11 @@
         <v>19</v>
       </c>
       <c r="B4" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A4)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A4)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A4)</f>
         <v>225000</v>
       </c>
     </row>
@@ -3535,11 +3753,11 @@
         <v>20</v>
       </c>
       <c r="B5" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A5)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A5)</f>
         <v>2</v>
       </c>
       <c r="C5" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A5)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A5)</f>
         <v>104200</v>
       </c>
     </row>
@@ -3548,11 +3766,11 @@
         <v>44</v>
       </c>
       <c r="B6" s="67">
-        <f>SUMIFS(Inventario!C3:C65,Inventario!A3:A65,A6)</f>
+        <f>SUMIFS(Inventario!C3:C70,Inventario!A3:A70,A6)</f>
         <v>2</v>
       </c>
       <c r="C6" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A6)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A6)</f>
         <v>80000</v>
       </c>
     </row>
@@ -3561,11 +3779,11 @@
         <v>21</v>
       </c>
       <c r="B7" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A7)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A7)</f>
         <v>4</v>
       </c>
       <c r="C7" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A7)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A7)</f>
         <v>300000</v>
       </c>
     </row>
@@ -3574,11 +3792,11 @@
         <v>22</v>
       </c>
       <c r="B8" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A8)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A8)</f>
         <v>2</v>
       </c>
       <c r="C8" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A8)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A8)</f>
         <v>110000</v>
       </c>
     </row>
@@ -3587,11 +3805,11 @@
         <v>23</v>
       </c>
       <c r="B9" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A9)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A9)</f>
         <v>3</v>
       </c>
       <c r="C9" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A9)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A9)</f>
         <v>225000</v>
       </c>
     </row>
@@ -3600,11 +3818,11 @@
         <v>24</v>
       </c>
       <c r="B10" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A10)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A10)</f>
         <v>2</v>
       </c>
       <c r="C10" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A10)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A10)</f>
         <v>110000</v>
       </c>
     </row>
@@ -3613,11 +3831,11 @@
         <v>25</v>
       </c>
       <c r="B11" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A11)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A11)</f>
         <v>10</v>
       </c>
       <c r="C11" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A11)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A11)</f>
         <v>750000</v>
       </c>
     </row>
@@ -3626,11 +3844,11 @@
         <v>26</v>
       </c>
       <c r="B12" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A12)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A12)</f>
         <v>1</v>
       </c>
       <c r="C12" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A12)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A12)</f>
         <v>50000</v>
       </c>
     </row>
@@ -3639,11 +3857,11 @@
         <v>27</v>
       </c>
       <c r="B13" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A13)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A13)</f>
         <v>11</v>
       </c>
       <c r="C13" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A13)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A13)</f>
         <v>622897</v>
       </c>
     </row>
@@ -3652,11 +3870,11 @@
         <v>29</v>
       </c>
       <c r="B14" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A14)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A14)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A14)</f>
         <v>39000</v>
       </c>
     </row>
@@ -3665,11 +3883,11 @@
         <v>30</v>
       </c>
       <c r="B15" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A15)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A15)</f>
         <v>0</v>
       </c>
       <c r="C15" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A15)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A15)</f>
         <v>0</v>
       </c>
     </row>
@@ -3678,11 +3896,11 @@
         <v>34</v>
       </c>
       <c r="B16" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A16)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A16)</f>
         <v>9</v>
       </c>
       <c r="C16" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A16)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A16)</f>
         <v>315000</v>
       </c>
     </row>
@@ -3691,11 +3909,11 @@
         <v>36</v>
       </c>
       <c r="B17" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A17)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A17)</f>
         <v>5</v>
       </c>
       <c r="C17" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A17)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A17)</f>
         <v>175000</v>
       </c>
     </row>
@@ -3704,11 +3922,11 @@
         <v>37</v>
       </c>
       <c r="B18" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A18)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A18)</f>
         <v>2</v>
       </c>
       <c r="C18" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A18)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A18)</f>
         <v>68000</v>
       </c>
     </row>
@@ -3717,11 +3935,11 @@
         <v>38</v>
       </c>
       <c r="B19" s="67">
-        <f>SUMIFS(Inventario!C2:C64,Inventario!A2:A64,A19)</f>
+        <f>SUMIFS(Inventario!C2:C69,Inventario!A2:A69,A19)</f>
         <v>4</v>
       </c>
       <c r="C19" s="6">
-        <f>SUMIFS(Inventario!$K$2:$K$64,Inventario!$A$2:$A$64,A19)</f>
+        <f>SUMIFS(Inventario!$K$2:$K$69,Inventario!$A$2:$A$69,A19)</f>
         <v>140000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
actulizandp catalogo polo albaricoque
</commit_message>
<xml_diff>
--- a/Inventario_CJ.xlsx
+++ b/Inventario_CJ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/463e7e6710c11b9a/Algoritmos/negocio de CJ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7147CD00-2E01-4A9F-9135-DD6FF5C83A0E}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="11_32D7F77174205C2ECD3847EFE09E77DAE5544094" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EB36D48-4D6F-4477-923F-CA6B78DD1EA4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="464" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3277,6 +3277,9 @@
       <c r="E60" s="69">
         <v>25000</v>
       </c>
+      <c r="F60" s="5">
+        <v>60000</v>
+      </c>
       <c r="G60" s="6">
         <f t="shared" ref="G60:G66" si="14">IF(AND(E60&lt;&gt;"",F61&lt;&gt;""),F61-E60,"")</f>
         <v>35000</v>

</xml_diff>